<commit_message>
B2 listening y speaking: práctica examen, audios, fotos y acceso alumnos.
Listening partes 10-13 con audios por ítem, scripts SQL/Excel y importación Supabase.
Speaking partes 14-17 con TTS, visualizador de voz y fotos long turn por examen.
Habilita Listening y Speaking en el menú B2 para todos los roles.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Ejercicios/Levels/B2/PARTE 10/Script para tabla levels_preguntas partes 10, 11,12 y 13.xlsx
+++ b/Ejercicios/Levels/B2/PARTE 10/Script para tabla levels_preguntas partes 10, 11,12 y 13.xlsx
@@ -1,18 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Charly\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Webs\english-practice\Ejercicios\Levels\B2\PARTE 10\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1322A43-D9C4-4408-A8F4-F554DF6A26EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Examen 1" sheetId="1" r:id="rId1"/>
+    <sheet name="examen 2,3,4 y 5" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="36">
   <si>
     <t>id</t>
   </si>
@@ -877,7 +879,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1194,7 +1196,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B4:G24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1506,4 +1508,37 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63382BBD-2C3F-43E5-BD84-C3791B9566E6}">
+  <dimension ref="A4:F4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="6" width="42.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>